<commit_message>
- updated figure 3A x title text format - updated stylistic changes of text in supplementary - updated abbreviation dictionary in supplementary - added full exclusion double check of TTBNP
</commit_message>
<xml_diff>
--- a/Outputs/Tables/T3.xlsx
+++ b/Outputs/Tables/T3.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="134">
   <si>
     <t xml:space="preserve">Chemical Name</t>
   </si>
@@ -146,6 +146,9 @@
     <t xml:space="preserve">-0.50ᵇ</t>
   </si>
   <si>
+    <t xml:space="preserve">0.010</t>
+  </si>
+  <si>
     <t xml:space="preserve">Acetophenone</t>
   </si>
   <si>
@@ -290,6 +293,15 @@
     <t xml:space="preserve">0.031</t>
   </si>
   <si>
+    <t xml:space="preserve">Dibutyl phthalate‡¶</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.035</t>
+  </si>
+  <si>
     <t xml:space="preserve">5-NOT†</t>
   </si>
   <si>
@@ -299,19 +311,10 @@
     <t xml:space="preserve">0.21ᵃ</t>
   </si>
   <si>
-    <t xml:space="preserve">0.035</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dibutyl phthalate‡¶</t>
-  </si>
-  <si>
-    <t xml:space="preserve">45%</t>
+    <t xml:space="preserve">0.036</t>
   </si>
   <si>
     <t xml:space="preserve">2,4'-Methoxychlor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.036</t>
   </si>
   <si>
     <t xml:space="preserve">o-Aminoazotoluene†‡¶</t>
@@ -961,18 +964,18 @@
         <v>43</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>8</v>
@@ -981,72 +984,72 @@
         <v>26</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>7</v>
@@ -1058,95 +1061,95 @@
         <v>26</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>83</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>13</v>
@@ -1161,44 +1164,44 @@
         <v>9</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>93</v>
+        <v>47</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>94</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>95</v>
@@ -1209,24 +1212,24 @@
         <v>96</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>46</v>
+        <v>97</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>7</v>
@@ -1246,13 +1249,13 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>14</v>
@@ -1261,15 +1264,15 @@
         <v>9</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>8</v>
@@ -1281,132 +1284,132 @@
         <v>16</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>8</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
@@ -1416,7 +1419,7 @@
     </row>
     <row r="32" ht="100" customHeight="1">
       <c r="A32" s="4" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>

</xml_diff>